<commit_message>
Tests actualizados: cartas y soporte
</commit_message>
<xml_diff>
--- a/Web/TestCases/Cartas.xlsx
+++ b/Web/TestCases/Cartas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nerea QA\PycharmProjects\KOVAI\Web\TestCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A21CD18-D164-48D4-B558-C8A6DF45455E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43F122E6-F105-4640-AD57-AC2DD17C3B59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1185" yWindow="4140" windowWidth="26415" windowHeight="12435" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="49">
   <si>
     <t>Num</t>
   </si>
@@ -65,9 +65,6 @@
   </si>
   <si>
     <t>KO</t>
-  </si>
-  <si>
-    <t>al dar a añadir carta no hace nada. Tampoco se ha podido añadir producto, si ese es el motivo u  otro error, falta mensaje de error explicativo.</t>
   </si>
   <si>
     <t>1. The user clicks "Escanear Carta con IA"
@@ -182,6 +179,9 @@
   </si>
   <si>
     <t>No se muestran restaurantes</t>
+  </si>
+  <si>
+    <t>Al dar a añadir carta no hace nada. Tampoco se ha podido añadir producto, si ese es el motivo u  otro error, falta mensaje de error explicativo.</t>
   </si>
 </sst>
 </file>
@@ -303,7 +303,7 @@
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="4">
     <dxf>
       <fill>
         <patternFill>
@@ -315,71 +315,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6565"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6565"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6565"/>
         </patternFill>
       </fill>
     </dxf>
@@ -750,16 +685,16 @@
         <v>8</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="F2" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G2" s="4" t="s">
         <v>12</v>
@@ -774,22 +709,22 @@
         <v>9</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>21</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>14</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>15</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:8" s="3" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -800,16 +735,16 @@
         <v>10</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>26</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>14</v>
@@ -826,16 +761,16 @@
         <v>10</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>18</v>
-      </c>
       <c r="F5" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>12</v>
@@ -850,16 +785,16 @@
         <v>11</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>12</v>
@@ -871,25 +806,25 @@
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>32</v>
       </c>
       <c r="G7" s="4" t="s">
         <v>14</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:8" s="3" customFormat="1" ht="60" x14ac:dyDescent="0.25">
@@ -897,25 +832,25 @@
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="D8" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="E8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="E8" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="G8" s="4" t="s">
+      <c r="H8" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:8" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -923,23 +858,23 @@
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="D9" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="E9" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>46</v>
       </c>
       <c r="F9" s="1"/>
       <c r="G9" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="H9" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -951,15 +886,15 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="G2:G9">
-    <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="KO">
+    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="KO">
       <formula>NOT(ISERROR(SEARCH("KO",G2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="5" priority="5" operator="containsText" text="OK">
+    <cfRule type="containsText" dxfId="2" priority="5" operator="containsText" text="OK">
       <formula>NOT(ISERROR(SEARCH("OK",G2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G8:G9">
-    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="BL">
+    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="BL">
       <formula>NOT(ISERROR(SEARCH("BL",G8)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>